<commit_message>
Update project documentation and submission file with optimization changes and corrected answers
</commit_message>
<xml_diff>
--- a/Calculations.xlsx
+++ b/Calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1a694778ec1de25c/Documentos/CE-321-Winter-2026-Project-3/CE_321_Project_3_Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="518" documentId="11_F25DC773A252ABDACC104835919973505ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85381423-A79C-47CB-A1A6-5F3D182365A2}"/>
+  <xr:revisionPtr revIDLastSave="549" documentId="11_F25DC773A252ABDACC104835919973505ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC76A7F4-FD66-491B-9303-3BD0F90CFA23}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="301">
   <si>
     <t>V_n</t>
   </si>
@@ -959,6 +959,9 @@
   </si>
   <si>
     <t>Do when ansers are verified, use code</t>
+  </si>
+  <si>
+    <t>*Or  11 3 3/4</t>
   </si>
 </sst>
 </file>
@@ -1355,17 +1358,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:M139"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1382,7 +1385,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1396,7 +1399,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1408,7 +1411,7 @@
       </c>
       <c r="F4">
         <f>(C12-25)/(5)*(H4-G4)+G4</f>
-        <v>0.94524999999999992</v>
+        <v>0.94</v>
       </c>
       <c r="G4">
         <v>0.94</v>
@@ -1417,7 +1420,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
@@ -1437,7 +1440,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1457,7 +1460,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B7" s="15" t="s">
         <v>6</v>
       </c>
@@ -1465,13 +1468,13 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B8" s="15"/>
       <c r="C8" s="1">
         <v>-0.18</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1485,7 +1488,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1493,8 +1496,7 @@
         <v>12</v>
       </c>
       <c r="C12" s="4">
-        <f>C11+(11+(3+3/4)/12)/2</f>
-        <v>25.65625</v>
+        <v>25</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>9</v>
@@ -1502,12 +1504,15 @@
       <c r="E12" t="s">
         <v>10</v>
       </c>
+      <c r="F12" t="s">
+        <v>300</v>
+      </c>
       <c r="I12" s="6" t="s">
         <v>48</v>
       </c>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1528,7 +1533,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1549,7 +1554,7 @@
         <v>-0.3</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1558,13 +1563,13 @@
       </c>
       <c r="C15" s="4">
         <f>0.00256*F4*C3*C4*C5*C2^2</f>
-        <v>32.002383999999999</v>
+        <v>31.824639999999999</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1586,7 +1591,7 @@
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1594,8 +1599,8 @@
         <v>37</v>
       </c>
       <c r="C17" s="4">
-        <f>C11/F5</f>
-        <v>0.41666666666666669</v>
+        <f>C12/F5</f>
+        <v>0.52083333333333337</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>9</v>
@@ -1612,7 +1617,7 @@
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -1621,7 +1626,7 @@
       </c>
       <c r="C18" s="4">
         <f>ATAN((C12-C11)*2/(F5/2))*180/PI()</f>
-        <v>25.237041255810915</v>
+        <v>22.619864948040426</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>39</v>
@@ -1631,7 +1636,7 @@
       </c>
       <c r="I18" s="10">
         <f>C17</f>
-        <v>0.41666666666666669</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="J18" s="8">
         <v>-0.2</v>
@@ -1644,10 +1649,10 @@
       </c>
       <c r="M18" s="8">
         <f>(I18-J17)/(K17-J17)*(K18-J18)+J18</f>
-        <v>-0.26666666666666666</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+        <v>-0.30833333333333335</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1666,7 +1671,7 @@
       <c r="L19" s="8"/>
       <c r="M19" s="8"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -1692,7 +1697,7 @@
       <c r="L20" s="8"/>
       <c r="M20" s="8"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -1707,7 +1712,7 @@
       </c>
       <c r="I21" s="10">
         <f>I18</f>
-        <v>0.41666666666666669</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="J21" s="8">
         <v>-0.2</v>
@@ -1723,7 +1728,7 @@
         <v>-0.2</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1732,13 +1737,13 @@
       </c>
       <c r="C22" s="4">
         <f>(C18-L18)/(L21-L18)*(M21-M18)+M18</f>
-        <v>-0.26350611658918782</v>
+        <v>-0.35990292612579078</v>
       </c>
       <c r="E22" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -1752,7 +1757,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -1761,14 +1766,14 @@
       </c>
       <c r="C24" s="4">
         <f>C15*C7</f>
-        <v>5.7604291199999995</v>
+        <v>5.7284351999999998</v>
       </c>
       <c r="D24" s="4">
         <f>C15*C8</f>
-        <v>-5.7604291199999995</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+        <v>-5.7284351999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1777,17 +1782,17 @@
       </c>
       <c r="C25" s="4">
         <f>C13*C6*(C19)-C24</f>
-        <v>13.808338880000003</v>
+        <v>13.840332800000002</v>
       </c>
       <c r="D25" s="11">
         <f>C13*C6*(C19)-D24</f>
-        <v>25.329197120000003</v>
+        <v>25.297203200000002</v>
       </c>
       <c r="E25" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>56</v>
       </c>
@@ -1796,17 +1801,17 @@
       </c>
       <c r="C26" s="4">
         <f>C14*C6*(C19)-C24</f>
-        <v>14.959442880000003</v>
+        <v>14.991436800000002</v>
       </c>
       <c r="D26" s="11">
         <f>C14*C6*(C19)-D24</f>
-        <v>26.48030112</v>
+        <v>26.448307200000002</v>
       </c>
       <c r="E26" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>57</v>
       </c>
@@ -1814,18 +1819,18 @@
         <v>43</v>
       </c>
       <c r="C27" s="4">
-        <f>C15*C8*(C20)-C24</f>
-        <v>-3.1106317247999997</v>
+        <f>C15*C6*(C20)-C24</f>
+        <v>-18.171869440000002</v>
       </c>
       <c r="D27" s="11">
-        <f>C15*C8*(C20)-D24</f>
-        <v>8.4102265151999998</v>
+        <f>C15*C6*(C20)-D24</f>
+        <v>-6.7149990400000004</v>
       </c>
       <c r="E27" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>58</v>
       </c>
@@ -1833,18 +1838,18 @@
         <v>71</v>
       </c>
       <c r="C28" s="4">
-        <f>C15*C8*(C21)-C24</f>
-        <v>-1.7281287360000004</v>
+        <f>C15*C6*(C21)-C24</f>
+        <v>-24.664095999999997</v>
       </c>
       <c r="D28" s="11">
-        <f>C15*C8*(C21)-D24</f>
-        <v>9.7927295039999986</v>
+        <f>C15*C6*(C21)-D24</f>
+        <v>-13.207225599999997</v>
       </c>
       <c r="E28" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -1852,18 +1857,18 @@
         <v>72</v>
       </c>
       <c r="C29" s="4">
-        <f>C15*C8*(C22)-C24</f>
-        <v>-4.2425208127015273</v>
+        <f>C15*C6*(C22)-C24</f>
+        <v>-15.464149100064903</v>
       </c>
       <c r="D29" s="11">
-        <f>C15*C8*(C22)-D24</f>
-        <v>7.2783374272984718</v>
+        <f>C15*C6*(C22)-D24</f>
+        <v>-4.0072787000649033</v>
       </c>
       <c r="E29" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>60</v>
       </c>
@@ -1871,18 +1876,18 @@
         <v>73</v>
       </c>
       <c r="C30" s="4">
-        <f>C15*C8*(C23)-C24</f>
-        <v>-2.3041716480000001</v>
+        <f>C15*C6*(C23)-C24</f>
+        <v>-21.959001599999997</v>
       </c>
       <c r="D30" s="11">
-        <f>C15*C8*(C23)-D24</f>
-        <v>9.2166865919999985</v>
+        <f>C15*C6*(C23)-D24</f>
+        <v>-10.502131199999997</v>
       </c>
       <c r="E30" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -1890,7 +1895,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -1905,7 +1910,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>63</v>
       </c>
@@ -1914,17 +1919,17 @@
       </c>
       <c r="C33" s="4">
         <f>$F$6/2*C25</f>
-        <v>276.16677760000005</v>
+        <v>276.80665600000003</v>
       </c>
       <c r="D33" s="4">
         <f>$F$6/2*D25</f>
-        <v>506.58394240000007</v>
+        <v>505.94406400000003</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>64</v>
       </c>
@@ -1933,17 +1938,17 @@
       </c>
       <c r="C34" s="4">
         <f>$F$6/2*C26</f>
-        <v>299.18885760000006</v>
+        <v>299.82873600000005</v>
       </c>
       <c r="D34" s="4">
         <f>F6/2*D26</f>
-        <v>529.60602240000003</v>
+        <v>528.96614399999999</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -1952,17 +1957,17 @@
       </c>
       <c r="C35" s="4">
         <f>$F$6/2*C27</f>
-        <v>-62.212634495999993</v>
+        <v>-363.43738880000001</v>
       </c>
       <c r="D35" s="4">
         <f>F6/2*D27</f>
-        <v>168.204530304</v>
+        <v>-134.29998080000001</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>66</v>
       </c>
@@ -1970,18 +1975,18 @@
         <v>80</v>
       </c>
       <c r="C36" s="4">
-        <f>$F$6/2*C28</f>
-        <v>-34.562574720000008</v>
+        <f>$F$6/2*C29</f>
+        <v>-309.28298200129808</v>
       </c>
       <c r="D36" s="4">
         <f>D29*F6/2</f>
-        <v>145.56674854596943</v>
+        <v>-80.145574001298058</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>67</v>
       </c>
@@ -1989,18 +1994,18 @@
         <v>81</v>
       </c>
       <c r="C37" s="4">
-        <f>$F$6/2*C29</f>
-        <v>-84.850416254030549</v>
+        <f>$F$6/2*C30</f>
+        <v>-439.18003199999993</v>
       </c>
       <c r="D37" s="4">
         <f>D30*F6/2</f>
-        <v>184.33373183999998</v>
+        <v>-210.04262399999993</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>68</v>
       </c>
@@ -2008,7 +2013,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>69</v>
       </c>
@@ -2016,7 +2021,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>83</v>
       </c>
@@ -2027,7 +2032,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -2035,7 +2040,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>85</v>
       </c>
@@ -2050,7 +2055,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>86</v>
       </c>
@@ -2065,7 +2070,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>87</v>
       </c>
@@ -2080,22 +2085,26 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>88</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C45" s="4">
+      <c r="C45" s="1">
+        <f>D45/2</f>
+        <v>4.423665364583333</v>
+      </c>
+      <c r="D45" s="4">
         <f>Proj1!C12/(Sheet1!$F$6/2)</f>
         <v>8.8473307291666661</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="E45" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>89</v>
       </c>
@@ -2104,13 +2113,13 @@
       </c>
       <c r="C46" s="4">
         <f>$C$36*C42</f>
-        <v>-148.21291603968754</v>
+        <v>-1326.2823448548504</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>90</v>
       </c>
@@ -2119,13 +2128,13 @@
       </c>
       <c r="C47" s="4">
         <f>$C$36*C43</f>
-        <v>-296.42583207937508</v>
+        <v>-2652.5646897097008</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>91</v>
       </c>
@@ -2134,13 +2143,13 @@
       </c>
       <c r="C48" s="4">
         <f>$C$36*C44</f>
-        <v>-301.10618073937508</v>
+        <v>-2694.4467601890433</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>92</v>
       </c>
@@ -2149,13 +2158,13 @@
       </c>
       <c r="C49" s="4">
         <f>$C$36*C45</f>
-        <v>-305.78652939937507</v>
+        <v>-1368.1644153341927</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>93</v>
       </c>
@@ -2164,13 +2173,13 @@
       </c>
       <c r="C50" s="4">
         <f>C37*C45</f>
-        <v>-750.69969510686724</v>
+        <v>-1942.7854963749996</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>94</v>
       </c>
@@ -2179,13 +2188,13 @@
       </c>
       <c r="C51" s="4">
         <f>C37*C44</f>
-        <v>-739.20953457246731</v>
+        <v>-3826.0986967499994</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>95</v>
       </c>
@@ -2194,13 +2203,13 @@
       </c>
       <c r="C52" s="4">
         <f>C37*C43</f>
-        <v>-727.71937403806737</v>
+        <v>-3766.6264007499994</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>96</v>
       </c>
@@ -2209,13 +2218,13 @@
       </c>
       <c r="C53" s="4">
         <f>C37*C42</f>
-        <v>-363.85968701903369</v>
+        <v>-1883.3132003749997</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>97</v>
       </c>
@@ -2223,7 +2232,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -2235,7 +2244,7 @@
         <v>637.4013671875</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>99</v>
       </c>
@@ -2246,7 +2255,7 @@
         <v>1074.802734375</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>100</v>
       </c>
@@ -2257,7 +2266,7 @@
         <v>1088.615234375</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>101</v>
       </c>
@@ -2268,7 +2277,7 @@
         <v>1302.427734375</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>102</v>
       </c>
@@ -2280,7 +2289,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>103</v>
       </c>
@@ -2292,7 +2301,7 @@
         <v>2097.916666666667</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>104</v>
       </c>
@@ -2303,7 +2312,7 @@
         <v>4195.8333333333339</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>105</v>
       </c>
@@ -2314,7 +2323,7 @@
         <v>4262.083333333333</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>106</v>
       </c>
@@ -2325,7 +2334,7 @@
         <v>4328.333333333333</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>107</v>
       </c>
@@ -2334,10 +2343,10 @@
       </c>
       <c r="C64" s="4">
         <f>SIN(C18*PI()/180)</f>
-        <v>0.42636416588259596</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.38461538461538458</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>108</v>
       </c>
@@ -2346,10 +2355,10 @@
       </c>
       <c r="C65" s="4">
         <f>COS(C18*PI()/180)</f>
-        <v>0.90455160054650185</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.92307692307692313</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>109</v>
       </c>
@@ -2358,13 +2367,13 @@
       </c>
       <c r="C66" s="4">
         <f>C46*C64</f>
-        <v>-63.192676320288605</v>
+        <v>-510.10859417494243</v>
       </c>
       <c r="F66" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>110</v>
       </c>
@@ -2372,8 +2381,8 @@
         <v>203</v>
       </c>
       <c r="C67" s="4">
-        <f>C55*G67+C59*G68+C46*C65*G69+C60*G70</f>
-        <v>2329.7737435329695</v>
+        <f>-(C55*G67+C59*G68+C46*C65*G69+C60*G70)</f>
+        <v>-1239.5793479384713</v>
       </c>
       <c r="F67" t="s">
         <v>224</v>
@@ -2382,7 +2391,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>111</v>
       </c>
@@ -2391,7 +2400,7 @@
       </c>
       <c r="C68" s="4">
         <f>C47*C64</f>
-        <v>-126.38535264057721</v>
+        <v>-1020.2171883498849</v>
       </c>
       <c r="F68" t="s">
         <v>225</v>
@@ -2400,7 +2409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>112</v>
       </c>
@@ -2408,8 +2417,8 @@
         <v>205</v>
       </c>
       <c r="C69" s="4">
-        <f>C56*G67+C59*G68+C47*G69*C65+C61*G70</f>
-        <v>3769.5474870659395</v>
+        <f>-(C56*G67+C59*G68+C47*G69*C65+C61*G70)</f>
+        <v>-1589.1586958769428</v>
       </c>
       <c r="F69" t="s">
         <v>226</v>
@@ -2418,7 +2427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>113</v>
       </c>
@@ -2427,7 +2436,7 @@
       </c>
       <c r="C70" s="4">
         <f>C48*C64</f>
-        <v>-128.38088559303785</v>
+        <v>-1036.3256769957859</v>
       </c>
       <c r="F70" t="s">
         <v>227</v>
@@ -2436,7 +2445,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>114</v>
       </c>
@@ -2444,11 +2453,11 @@
         <v>207</v>
       </c>
       <c r="C71" s="4">
-        <f>C57*G67+C59*G68+C48*C65*G69+C62*G70</f>
-        <v>3815.0138701944206</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+        <f>-(C57*G67+C59*G68+C48*C65*G69+C62*G70)</f>
+        <v>-1600.19832312678</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>115</v>
       </c>
@@ -2457,10 +2466,10 @@
       </c>
       <c r="C72" s="4">
         <f>C49*C64-C64*C50</f>
-        <v>189.69503078706006</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+        <v>221.00810809261804</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>216</v>
       </c>
@@ -2468,11 +2477,11 @@
         <v>209</v>
       </c>
       <c r="C73" s="4">
-        <f>C58*G67+C59*G68+C49*C65*G69+C50*C65*G69+C63*G70</f>
-        <v>3421.4336425842143</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+        <f>-(C58*G67+C59*G68+C49*C65*G69+C50*C65*G69+C63*G70)</f>
+        <v>-1320.8184909543352</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>217</v>
       </c>
@@ -2481,10 +2490,10 @@
       </c>
       <c r="C74" s="4">
         <f>-C64*C51</f>
-        <v>315.17245662045201</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1471.5764218269228</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>218</v>
       </c>
@@ -2492,11 +2501,11 @@
         <v>211</v>
       </c>
       <c r="C75" s="4">
-        <f>C57*G67+C59*G68+C51*C65*G69+C62*G70</f>
-        <v>3418.7267802799065</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+        <f>-(C57*G67+C59*G68+C51*C65*G69+C62*G70)</f>
+        <v>-555.59653553205135</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>219</v>
       </c>
@@ -2505,10 +2514,10 @@
       </c>
       <c r="C76" s="4">
         <f>-C64*C52</f>
-        <v>310.27346390834543</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1448.7024618269227</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>220</v>
       </c>
@@ -2516,11 +2525,11 @@
         <v>213</v>
       </c>
       <c r="C77" s="4">
-        <f>C56*G67+C59*G68+C52*C65*G69+G70*C61</f>
-        <v>3379.4202233818346</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+        <f>-(C56*G67+C59*G68+C52*C65*G69+G70*C61)</f>
+        <v>-560.79403953205178</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>221</v>
       </c>
@@ -2529,10 +2538,10 @@
       </c>
       <c r="C78" s="4">
         <f>-C64*C53</f>
-        <v>155.13673195417272</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+        <v>724.35123091346134</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>222</v>
       </c>
@@ -2540,11 +2549,11 @@
         <v>215</v>
       </c>
       <c r="C79" s="4">
-        <f>C55*G67+C59*G68+C65*C53*G69+G70*C60</f>
-        <v>2134.7101116909171</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+        <f>-(C55*G67+C59*G68+C65*C53*G69+G70*C60)</f>
+        <v>-725.39701976602578</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>228</v>
       </c>
@@ -2552,7 +2561,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>229</v>
       </c>
@@ -2563,7 +2572,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>231</v>
       </c>
@@ -2574,7 +2583,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>232</v>
       </c>
@@ -2585,7 +2594,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>233</v>
       </c>
@@ -2596,7 +2605,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>234</v>
       </c>
@@ -2607,7 +2616,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>235</v>
       </c>
@@ -2618,7 +2627,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>236</v>
       </c>
@@ -2629,7 +2638,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>237</v>
       </c>
@@ -2640,7 +2649,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>238</v>
       </c>
@@ -2651,7 +2660,7 @@
         <v>-0.22800000000000001</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>239</v>
       </c>
@@ -2662,7 +2671,7 @@
         <v>5.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>240</v>
       </c>
@@ -2673,7 +2682,7 @@
         <v>-0.23100000000000001</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>241</v>
       </c>
@@ -2681,7 +2690,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>242</v>
       </c>
@@ -2689,7 +2698,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>243</v>
       </c>
@@ -2697,7 +2706,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>244</v>
       </c>
@@ -2705,222 +2714,222 @@
         <v>74</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>288</v>
       </c>
@@ -2941,10 +2950,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{634D6E1C-9FE4-4600-90DE-E413A2AD2021}">
   <dimension ref="B2:K80"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="13" t="s">
         <v>117</v>
       </c>
@@ -2974,7 +2983,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B4" s="13" t="s">
         <v>121</v>
       </c>
@@ -3004,7 +3013,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="13" t="s">
         <v>124</v>
       </c>
@@ -3025,7 +3034,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" s="13" t="s">
         <v>126</v>
       </c>
@@ -3046,7 +3055,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
       <c r="I7" s="13" t="s">
         <v>128</v>
       </c>
@@ -3058,7 +3067,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
         <v>129</v>
       </c>
@@ -3076,7 +3085,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B9" s="13" t="s">
         <v>132</v>
       </c>
@@ -3102,7 +3111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B10" s="13" t="s">
         <v>134</v>
       </c>
@@ -3128,7 +3137,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B11" s="13" t="s">
         <v>136</v>
       </c>
@@ -3154,7 +3163,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>138</v>
       </c>
@@ -3180,7 +3189,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.3">
       <c r="I13" s="13" t="s">
         <v>140</v>
       </c>
@@ -3191,7 +3200,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B14" s="13" t="s">
         <v>141</v>
       </c>
@@ -3208,7 +3217,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B15" s="13" t="s">
         <v>132</v>
       </c>
@@ -3234,7 +3243,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B16" s="13" t="s">
         <v>134</v>
       </c>
@@ -3250,7 +3259,7 @@
         <v>4195.8333333333339</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
         <v>136</v>
       </c>
@@ -3266,7 +3275,7 @@
         <v>4262.083333333333</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="13" t="s">
         <v>138</v>
       </c>
@@ -3282,8 +3291,8 @@
         <v>4328.333333333333</v>
       </c>
     </row>
-    <row r="19" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="13" t="s">
         <v>146</v>
       </c>
@@ -3291,7 +3300,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>132</v>
       </c>
@@ -3306,7 +3315,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="13" t="s">
         <v>134</v>
       </c>
@@ -3321,7 +3330,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="13" t="s">
         <v>136</v>
       </c>
@@ -3336,7 +3345,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="13" t="s">
         <v>138</v>
       </c>
@@ -3351,8 +3360,8 @@
         <v>650</v>
       </c>
     </row>
-    <row r="25" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="13" t="s">
         <v>148</v>
       </c>
@@ -3360,7 +3369,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="13" t="s">
         <v>132</v>
       </c>
@@ -3375,7 +3384,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="13" t="s">
         <v>134</v>
       </c>
@@ -3390,7 +3399,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="13" t="s">
         <v>136</v>
       </c>
@@ -3405,7 +3414,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="13" t="s">
         <v>138</v>
       </c>
@@ -3414,8 +3423,8 @@
         <v>1302.427734375</v>
       </c>
     </row>
-    <row r="31" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="13" t="s">
         <v>153</v>
       </c>
@@ -3426,7 +3435,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="13" t="s">
         <v>132</v>
       </c>
@@ -3442,7 +3451,7 @@
         <v>2853.8399739583333</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="13" t="s">
         <v>134</v>
       </c>
@@ -3458,7 +3467,7 @@
         <v>4427.6799479166666</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" s="13" t="s">
         <v>136</v>
       </c>
@@ -3474,7 +3483,7 @@
         <v>4477.3799479166664</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" s="13" t="s">
         <v>138</v>
       </c>
@@ -3490,8 +3499,8 @@
         <v>4767.0799479166662</v>
       </c>
     </row>
-    <row r="37" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="13" t="s">
         <v>155</v>
       </c>
@@ -3499,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B39" s="13" t="s">
         <v>156</v>
       </c>
@@ -3508,7 +3517,7 @@
         <v>14142.43984375</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B40" s="13" t="s">
         <v>157</v>
       </c>
@@ -3517,8 +3526,8 @@
         <v>14142.43984375</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B42" s="13" t="s">
         <v>158</v>
       </c>
@@ -3527,7 +3536,7 @@
         <v>-29351.696513313043</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="13" t="s">
         <v>159</v>
       </c>
@@ -3536,7 +3545,7 @@
         <v>27093.530922069807</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B44" s="13" t="s">
         <v>160</v>
       </c>
@@ -3545,7 +3554,7 @@
         <v>27093.530922069807</v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B45" s="13" t="s">
         <v>161</v>
       </c>
@@ -3553,7 +3562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B46" s="13" t="s">
         <v>162</v>
       </c>
@@ -3569,7 +3578,7 @@
         <v>0.7094432754186335</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B47" s="13" t="s">
         <v>164</v>
       </c>
@@ -3578,7 +3587,7 @@
         <v>-23614.560186425493</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B48" s="13" t="s">
         <v>165</v>
       </c>
@@ -3587,7 +3596,7 @@
         <v>-23614.560186425493</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B49" s="13" t="s">
         <v>166</v>
       </c>
@@ -3596,7 +3605,7 @@
         <v>-4477.3799479166664</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B50" s="13" t="s">
         <v>167</v>
       </c>
@@ -3605,7 +3614,7 @@
         <v>16339.285662829792</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B51" s="13" t="s">
         <v>168</v>
       </c>
@@ -3614,7 +3623,7 @@
         <v>8627.7626325162073</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B52" s="13" t="s">
         <v>140</v>
       </c>
@@ -3622,7 +3631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B53" s="13" t="s">
         <v>169</v>
       </c>
@@ -3631,7 +3640,7 @@
         <v>16339.285662829792</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B54" s="13" t="s">
         <v>170</v>
       </c>
@@ -3640,7 +3649,7 @@
         <v>-23614.560186425493</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B55" s="13" t="s">
         <v>171</v>
       </c>
@@ -3649,7 +3658,7 @@
         <v>8627.7626325162073</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B56" s="13" t="s">
         <v>172</v>
       </c>
@@ -3658,7 +3667,7 @@
         <v>-23614.560186425493</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B57" s="13" t="s">
         <v>173</v>
       </c>
@@ -3667,7 +3676,7 @@
         <v>-4477.3799479166664</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B58" s="13" t="s">
         <v>174</v>
       </c>
@@ -3676,7 +3685,7 @@
         <v>27093.530922069807</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B59" s="13" t="s">
         <v>175</v>
       </c>
@@ -3685,7 +3694,7 @@
         <v>-5737.1363268875502</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B60" s="13" t="s">
         <v>176</v>
       </c>
@@ -3694,7 +3703,7 @@
         <v>27093.530922069807</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B61" s="13" t="s">
         <v>177</v>
       </c>
@@ -3703,7 +3712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B62" s="13" t="s">
         <v>178</v>
       </c>
@@ -3712,24 +3721,24 @@
         <v>-29351.696513313043</v>
       </c>
     </row>
-    <row r="63" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="2:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>